<commit_message>
Video script: SugarAI is delivered, not created, by HLB HAMT
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BzGR1oZYiJrjuzjRzG6Qzk
</commit_message>
<xml_diff>
--- a/SugarAI_HLB_HAMT_60s_video_plan.xlsx
+++ b/SugarAI_HLB_HAMT_60s_video_plan.xlsx
@@ -580,7 +580,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>So we created SugarAI: one complete picture of every customer's journey.</t>
+          <t>So we bring you SugarAI: one complete picture of every customer's journey.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -883,7 +883,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>So we created SugarAI: one complete picture of every customer's journey.</t>
+          <t>So we bring you SugarAI: one complete picture of every customer's journey.</t>
         </is>
       </c>
     </row>

</xml_diff>